<commit_message>
Refactor validation and training scripts; update README for environment setup
- Updated README.md to clarify virtual environment activation for Windows and Mac.
- Refactored classificar.py to improve data handling and validation logic, including:
  - Cleaned up Excel headers and ensured proper data type conversion.
  - Enhanced forward pass logic for hidden and output layers.
  - Implemented binary filtering for output predictions.
- Modified pmc.py to streamline data extraction and training process, including:
  - Adjusted input and output dimensions for neural network.
  - Improved weight initialization and training loop with shuffling for better performance.
  - Updated result saving logic to reflect changes in output structure.
- Added new validation dataset and updated existing datasets.
- Updated graphics for error evolution during training.
</commit_message>
<xml_diff>
--- a/datasets/resultados.xlsx
+++ b/datasets/resultados.xlsx
@@ -413,21 +413,31 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Treinamentos</t>
+          <t>Treinamento</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
+          <t>MSE</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Epocas</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
           <t>erro-quadratico-medio</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Numero-de-epocas</t>
         </is>
@@ -436,53 +446,77 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>T1_x000d_</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.001518369512054261</v>
+        <v>0.05071057645120201</v>
       </c>
       <c r="C2" t="n">
-        <v>195</v>
+        <v>3000</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0.02793674416873917</v>
+      </c>
+      <c r="E2" t="n">
+        <v>2512</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>T2_x000d_</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.001487016525681273</v>
+        <v>0.03252858304552518</v>
       </c>
       <c r="C3" t="n">
-        <v>181</v>
+        <v>3000</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0.03364154403368873</v>
+      </c>
+      <c r="E3" t="n">
+        <v>351</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>T3_x000d_</t>
+          <t>T3</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.001439105349605169</v>
+        <v>0.01851913507430689</v>
       </c>
       <c r="C4" t="n">
-        <v>220</v>
+        <v>3000</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0.07092264598015992</v>
+      </c>
+      <c r="E4" t="n">
+        <v>156</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>T4_x000d_</t>
+          <t>T4</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.001502819046877044</v>
+        <v>0.03535144765374056</v>
       </c>
       <c r="C5" t="n">
-        <v>222</v>
+        <v>3000</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0.03158234908463897</v>
+      </c>
+      <c r="E5" t="n">
+        <v>461</v>
       </c>
     </row>
     <row r="6">
@@ -492,10 +526,16 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.001462028118042074</v>
+        <v>0.04207186680741264</v>
       </c>
       <c r="C6" t="n">
-        <v>245</v>
+        <v>3000</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0.0373263947217664</v>
+      </c>
+      <c r="E6" t="n">
+        <v>305</v>
       </c>
     </row>
   </sheetData>

</xml_diff>